<commit_message>
Completed dynamic monthly and quarterly report rendering
</commit_message>
<xml_diff>
--- a/data/sample_MOU_data.xlsx
+++ b/data/sample_MOU_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rames\OneDrive\Desktop\Projects\SalesReport\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62871A5B-57C1-4AC4-BE87-A8148385B951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B78B78EA-3A09-4A28-BD02-D9E44D8F4D2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="19515" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6060" yWindow="4860" windowWidth="19515" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -748,16 +748,16 @@
         <v>58</v>
       </c>
       <c r="C7">
+        <v>200000</v>
+      </c>
+      <c r="D7">
         <v>250000</v>
-      </c>
-      <c r="D7">
-        <v>235000</v>
       </c>
       <c r="E7">
         <v>15000</v>
       </c>
       <c r="F7">
-        <v>260000</v>
+        <v>200000</v>
       </c>
       <c r="G7">
         <v>252000</v>
@@ -766,25 +766,25 @@
         <v>8000</v>
       </c>
       <c r="I7">
-        <v>280000</v>
+        <v>200000</v>
       </c>
       <c r="J7">
-        <v>270000</v>
+        <v>180000</v>
       </c>
       <c r="K7">
         <v>10000</v>
       </c>
       <c r="L7">
-        <v>790000</v>
+        <v>600000</v>
       </c>
       <c r="M7">
-        <v>757000</v>
+        <v>682000</v>
       </c>
       <c r="N7">
         <v>33000</v>
       </c>
       <c r="O7">
-        <v>300000</v>
+        <v>200000</v>
       </c>
       <c r="P7">
         <v>295000</v>
@@ -892,16 +892,16 @@
         <v>12000</v>
       </c>
       <c r="AY7">
-        <v>3870000</v>
+        <v>2000000</v>
       </c>
       <c r="AZ7">
-        <v>3765000</v>
+        <v>1500000</v>
       </c>
       <c r="BA7">
         <v>105000</v>
       </c>
       <c r="BB7">
-        <v>97.29</v>
+        <v>75</v>
       </c>
       <c r="BC7" t="s">
         <v>59</v>

</xml_diff>